<commit_message>
Adjust NEW_STOCKS_REGISTRY masking logic to allow technical indicator calculation
Updated the apply_new_stocks_registry function in backtest_adj4_fixed.py to use constant-price masking instead of NaN masking. This ensures that stocks added to the pool in new quarters (like 3481) can calculate their 303-day SMA immediately upon their effective date, provided sufficient historical data exists in the raw dataset. The logic maintains historical integrity by setting ROC to 0 and Volume to 0 before the effective date.

Co-authored-by: lij1017-cmd <261091087+lij1017-cmd@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/trendstrategy_results_equityV-adj4-2-260616_fixed.xlsx
+++ b/trendstrategy_results_equityV-adj4-2-260616_fixed.xlsx
@@ -2851,7 +2851,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0.6666666666666666</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -2874,7 +2874,7 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>0.6590909090909091</v>
+        <v>0.6304347826086957</v>
       </c>
       <c r="F3">
         <v>11910</v>
@@ -2897,7 +2897,7 @@
         <v>-0.001238866666666667</v>
       </c>
       <c r="E4">
-        <v>0.6742424242424242</v>
+        <v>0.644927536231884</v>
       </c>
       <c r="F4">
         <v>-173920</v>
@@ -2920,7 +2920,7 @@
         <v>-0.001346666666666667</v>
       </c>
       <c r="E5">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F5">
         <v>-190090</v>
@@ -2943,7 +2943,7 @@
         <v>-0.0047262</v>
       </c>
       <c r="E6">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F6">
         <v>-697020</v>
@@ -2966,7 +2966,7 @@
         <v>-0.01267033333333333</v>
       </c>
       <c r="E7">
-        <v>0.7045454545454546</v>
+        <v>0.6739130434782609</v>
       </c>
       <c r="F7">
         <v>-1888640</v>
@@ -2989,7 +2989,7 @@
         <v>-0.002903072333333318</v>
       </c>
       <c r="E8">
-        <v>0.7196969696969697</v>
+        <v>0.6884057971014492</v>
       </c>
       <c r="F8">
         <v>-423550.8499999978</v>
@@ -3012,7 +3012,7 @@
         <v>-0.0007197395083333303</v>
       </c>
       <c r="E9">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F9">
         <v>-96050.92624999955</v>
@@ -3035,7 +3035,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F10">
         <v>670949.0737500004</v>
@@ -3058,7 +3058,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F11">
         <v>890949.0737500004</v>
@@ -3081,7 +3081,7 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>0.7045454545454546</v>
+        <v>0.6739130434782609</v>
       </c>
       <c r="F12">
         <v>1227949.07375</v>
@@ -3104,7 +3104,7 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>0.7045454545454546</v>
+        <v>0.6739130434782609</v>
       </c>
       <c r="F13">
         <v>2917949.07375</v>
@@ -3127,7 +3127,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>0.696969696969697</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F14">
         <v>3756949.07375</v>
@@ -3150,7 +3150,7 @@
         <v>-0.01561333333333333</v>
       </c>
       <c r="E15">
-        <v>0.6893939393939394</v>
+        <v>0.6594202898550725</v>
       </c>
       <c r="F15">
         <v>1414949.07375</v>
@@ -3173,7 +3173,7 @@
         <v>-0.007786666666666667</v>
       </c>
       <c r="E16">
-        <v>0.7045454545454546</v>
+        <v>0.6739130434782609</v>
       </c>
       <c r="F16">
         <v>2588949.07375</v>
@@ -3196,7 +3196,7 @@
         <v>-0.007633333333333333</v>
       </c>
       <c r="E17">
-        <v>0.696969696969697</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F17">
         <v>2611949.07375</v>
@@ -3219,7 +3219,7 @@
         <v>-0.0008084251333333552</v>
       </c>
       <c r="E18">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F18">
         <v>3635685.303749997</v>
@@ -3242,7 +3242,7 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F19">
         <v>4365485.303749997</v>
@@ -3265,7 +3265,7 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>0.7348484848484849</v>
+        <v>0.7028985507246377</v>
       </c>
       <c r="F20">
         <v>4713285.303749997</v>
@@ -3288,7 +3288,7 @@
         <v>-0.01188533333333333</v>
       </c>
       <c r="E21">
-        <v>0.7121212121212122</v>
+        <v>0.6811594202898551</v>
       </c>
       <c r="F21">
         <v>2930485.303749997</v>
@@ -3311,7 +3311,7 @@
         <v>-0.01391466666666667</v>
       </c>
       <c r="E22">
-        <v>0.6818181818181818</v>
+        <v>0.6521739130434783</v>
       </c>
       <c r="F22">
         <v>2626085.303749997</v>
@@ -3334,7 +3334,7 @@
         <v>-0.01766533333333333</v>
       </c>
       <c r="E23">
-        <v>0.6818181818181818</v>
+        <v>0.6521739130434783</v>
       </c>
       <c r="F23">
         <v>2063485.303749997</v>
@@ -3357,7 +3357,7 @@
         <v>-0.0103051463333333</v>
       </c>
       <c r="E24">
-        <v>0.6893939393939394</v>
+        <v>0.6594202898550725</v>
       </c>
       <c r="F24">
         <v>3167513.353750002</v>
@@ -3380,7 +3380,7 @@
         <v>-0.001230479666666637</v>
       </c>
       <c r="E25">
-        <v>0.6893939393939394</v>
+        <v>0.6594202898550725</v>
       </c>
       <c r="F25">
         <v>4528713.353750002</v>
@@ -3403,7 +3403,7 @@
         <v>-0.009085146333333304</v>
       </c>
       <c r="E26">
-        <v>0.696969696969697</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F26">
         <v>3350513.353750002</v>
@@ -3426,7 +3426,7 @@
         <v>-0.01165954949999998</v>
       </c>
       <c r="E27">
-        <v>0.6666666666666666</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="F27">
         <v>2964352.87875</v>
@@ -3449,7 +3449,7 @@
         <v>0</v>
       </c>
       <c r="E28">
-        <v>0.7045454545454546</v>
+        <v>0.6739130434782609</v>
       </c>
       <c r="F28">
         <v>4824352.87875</v>
@@ -3472,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>0.696969696969697</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F29">
         <v>5384352.87875</v>
@@ -3495,7 +3495,7 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>0.6893939393939394</v>
+        <v>0.6594202898550725</v>
       </c>
       <c r="F30">
         <v>6684352.87875</v>
@@ -3518,7 +3518,7 @@
         <v>0</v>
       </c>
       <c r="E31">
-        <v>0.6893939393939394</v>
+        <v>0.6594202898550725</v>
       </c>
       <c r="F31">
         <v>8284352.87875</v>
@@ -3541,7 +3541,7 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>0.7196969696969697</v>
+        <v>0.6884057971014492</v>
       </c>
       <c r="F32">
         <v>9854352.87875</v>
@@ -3564,7 +3564,7 @@
         <v>0</v>
       </c>
       <c r="E33">
-        <v>0.7272727272727273</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="F33">
         <v>11374352.87875</v>
@@ -3587,7 +3587,7 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>0.7348484848484849</v>
+        <v>0.7028985507246377</v>
       </c>
       <c r="F34">
         <v>11564352.87875</v>
@@ -3610,7 +3610,7 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>0.7575757575757576</v>
+        <v>0.7246376811594203</v>
       </c>
       <c r="F35">
         <v>12964352.87875</v>
@@ -3633,7 +3633,7 @@
         <v>-0.003768934666666687</v>
       </c>
       <c r="E36">
-        <v>0.7196969696969697</v>
+        <v>0.6884057971014492</v>
       </c>
       <c r="F36">
         <v>12399012.67875</v>
@@ -3656,7 +3656,7 @@
         <v>-0.02712893466666669</v>
       </c>
       <c r="E37">
-        <v>0.6287878787878788</v>
+        <v>0.6014492753623188</v>
       </c>
       <c r="F37">
         <v>8895012.678749997</v>
@@ -3679,7 +3679,7 @@
         <v>-0.03136893466666669</v>
       </c>
       <c r="E38">
-        <v>0.6893939393939394</v>
+        <v>0.6594202898550725</v>
       </c>
       <c r="F38">
         <v>8259012.678749997</v>
@@ -3702,7 +3702,7 @@
         <v>-0.03570476133333336</v>
       </c>
       <c r="E39">
-        <v>0.696969696969697</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F39">
         <v>7608638.678749997</v>
@@ -3725,7 +3725,7 @@
         <v>-0.05159809466666668</v>
       </c>
       <c r="E40">
-        <v>0.6136363636363636</v>
+        <v>0.5869565217391305</v>
       </c>
       <c r="F40">
         <v>5224638.678749997</v>
@@ -3748,7 +3748,7 @@
         <v>-0.04526442800000002</v>
       </c>
       <c r="E41">
-        <v>0.6363636363636364</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="F41">
         <v>6174688.678749997</v>
@@ -3771,7 +3771,7 @@
         <v>-0.03961109466666669</v>
       </c>
       <c r="E42">
-        <v>0.6742424242424242</v>
+        <v>0.644927536231884</v>
       </c>
       <c r="F42">
         <v>7022688.678749997</v>
@@ -3794,7 +3794,7 @@
         <v>-0.03555776133333335</v>
       </c>
       <c r="E43">
-        <v>0.6590909090909091</v>
+        <v>0.6304347826086957</v>
       </c>
       <c r="F43">
         <v>7630688.678749997</v>
@@ -3817,7 +3817,7 @@
         <v>-0.02915776133333335</v>
       </c>
       <c r="E44">
-        <v>0.6439393939393939</v>
+        <v>0.6159420289855072</v>
       </c>
       <c r="F44">
         <v>8590688.678749997</v>
@@ -3840,7 +3840,7 @@
         <v>-0.02421161133333335</v>
       </c>
       <c r="E45">
-        <v>0.6666666666666666</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="F45">
         <v>9332611.178749997</v>
@@ -3863,7 +3863,7 @@
         <v>-0.03411827800000002</v>
       </c>
       <c r="E46">
-        <v>0.696969696969697</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F46">
         <v>7846611.178749997</v>
@@ -3886,7 +3886,7 @@
         <v>-0.02782494466666669</v>
       </c>
       <c r="E47">
-        <v>0.696969696969697</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F47">
         <v>8790611.178749997</v>
@@ -3909,7 +3909,7 @@
         <v>-0.01982494466666669</v>
       </c>
       <c r="E48">
-        <v>0.6818181818181818</v>
+        <v>0.6521739130434783</v>
       </c>
       <c r="F48">
         <v>9990611.178749997</v>
@@ -3932,7 +3932,7 @@
         <v>-0.01273161133333335</v>
       </c>
       <c r="E49">
-        <v>0.6818181818181818</v>
+        <v>0.6521739130434783</v>
       </c>
       <c r="F49">
         <v>11054611.17875</v>
@@ -3955,7 +3955,7 @@
         <v>-0.02022494466666669</v>
       </c>
       <c r="E50">
-        <v>0.6515151515151515</v>
+        <v>0.6231884057971014</v>
       </c>
       <c r="F50">
         <v>9930611.178749997</v>
@@ -3978,7 +3978,7 @@
         <v>-0.01646494466666669</v>
       </c>
       <c r="E51">
-        <v>0.6590909090909091</v>
+        <v>0.6304347826086957</v>
       </c>
       <c r="F51">
         <v>10494611.17875</v>
@@ -4001,7 +4001,7 @@
         <v>0</v>
       </c>
       <c r="E52">
-        <v>0.6666666666666666</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="F52">
         <v>13330611.17875</v>
@@ -4024,7 +4024,7 @@
         <v>-0.00704</v>
       </c>
       <c r="E53">
-        <v>0.6666666666666666</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="F53">
         <v>12274611.17875</v>
@@ -4047,7 +4047,7 @@
         <v>-0.002671867666666607</v>
       </c>
       <c r="E54">
-        <v>0.6818181818181818</v>
+        <v>0.6521739130434783</v>
       </c>
       <c r="F54">
         <v>12929831.02875001</v>
@@ -4070,7 +4070,7 @@
         <v>-0.01075853433333327</v>
       </c>
       <c r="E55">
-        <v>0.6742424242424242</v>
+        <v>0.644927536231884</v>
       </c>
       <c r="F55">
         <v>11716831.02875001</v>
@@ -4093,7 +4093,7 @@
         <v>-0.03150520099999994</v>
       </c>
       <c r="E56">
-        <v>0.6363636363636364</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="F56">
         <v>8604831.028750006</v>
@@ -4139,7 +4139,7 @@
         <v>-0.008378534333333274</v>
       </c>
       <c r="E58">
-        <v>0.6304347826086957</v>
+        <v>0.6376811594202898</v>
       </c>
       <c r="F58">
         <v>12073831.02875001</v>
@@ -4162,7 +4162,7 @@
         <v>0</v>
       </c>
       <c r="E59">
-        <v>0.6231884057971014</v>
+        <v>0.644927536231884</v>
       </c>
       <c r="F59">
         <v>13643831.02875001</v>
@@ -4185,7 +4185,7 @@
         <v>0</v>
       </c>
       <c r="E60">
-        <v>0.6594202898550725</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="F60">
         <v>16688831.02875001</v>
@@ -4208,7 +4208,7 @@
         <v>-0.01886666666666667</v>
       </c>
       <c r="E61">
-        <v>0.6739130434782609</v>
+        <v>0.7028985507246377</v>
       </c>
       <c r="F61">
         <v>13858831.02875001</v>
@@ -4231,7 +4231,7 @@
         <v>0</v>
       </c>
       <c r="E62">
-        <v>0.6739130434782609</v>
+        <v>0.7101449275362319</v>
       </c>
       <c r="F62">
         <v>17141831.02875001</v>
@@ -4254,7 +4254,7 @@
         <v>0</v>
       </c>
       <c r="E63">
-        <v>0.6666666666666666</v>
+        <v>0.7101449275362319</v>
       </c>
       <c r="F63">
         <v>19754647.65375001</v>
@@ -4277,7 +4277,7 @@
         <v>-0.01</v>
       </c>
       <c r="E64">
-        <v>0.6956521739130435</v>
+        <v>0.7391304347826086</v>
       </c>
       <c r="F64">
         <v>18254647.65375001</v>
@@ -4300,7 +4300,7 @@
         <v>-0.01353333333333333</v>
       </c>
       <c r="E65">
-        <v>0.6956521739130435</v>
+        <v>0.7391304347826086</v>
       </c>
       <c r="F65">
         <v>17724647.65375001</v>
@@ -4323,7 +4323,7 @@
         <v>-0.008266666666666667</v>
       </c>
       <c r="E66">
-        <v>0.7028985507246377</v>
+        <v>0.7463768115942029</v>
       </c>
       <c r="F66">
         <v>18514647.65375001</v>
@@ -4346,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>0.7173913043478261</v>
+        <v>0.7536231884057971</v>
       </c>
       <c r="F67">
         <v>20259647.65375001</v>
@@ -4369,7 +4369,7 @@
         <v>0</v>
       </c>
       <c r="E68">
-        <v>0.7173913043478261</v>
+        <v>0.7536231884057971</v>
       </c>
       <c r="F68">
         <v>23094647.65375001</v>
@@ -4392,7 +4392,7 @@
         <v>0</v>
       </c>
       <c r="E69">
-        <v>0.7101449275362319</v>
+        <v>0.7536231884057971</v>
       </c>
       <c r="F69">
         <v>25344647.65375001</v>
@@ -4415,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="E70">
-        <v>0.7391304347826086</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="F70">
         <v>27259647.65375001</v>
@@ -4438,7 +4438,7 @@
         <v>0</v>
       </c>
       <c r="E71">
-        <v>0.7173913043478261</v>
+        <v>0.7391304347826086</v>
       </c>
       <c r="F71">
         <v>27289647.65375001</v>
@@ -4461,7 +4461,7 @@
         <v>0</v>
       </c>
       <c r="E72">
-        <v>0.7101449275362319</v>
+        <v>0.7391304347826086</v>
       </c>
       <c r="F72">
         <v>28755663.80375</v>
@@ -4484,7 +4484,7 @@
         <v>-0.02611</v>
       </c>
       <c r="E73">
-        <v>0.7101449275362319</v>
+        <v>0.7391304347826086</v>
       </c>
       <c r="F73">
         <v>24839163.80375</v>
@@ -4507,7 +4507,7 @@
         <v>-0.01577666666666667</v>
       </c>
       <c r="E74">
-        <v>0.6884057971014492</v>
+        <v>0.7173913043478261</v>
       </c>
       <c r="F74">
         <v>26389163.80375</v>
@@ -4530,7 +4530,7 @@
         <v>-0.005325176666666666</v>
       </c>
       <c r="E75">
-        <v>0.6956521739130435</v>
+        <v>0.7318840579710145</v>
       </c>
       <c r="F75">
         <v>27956887.30375</v>
@@ -4553,7 +4553,7 @@
         <v>-0.00119851</v>
       </c>
       <c r="E76">
-        <v>0.6884057971014492</v>
+        <v>0.7246376811594203</v>
       </c>
       <c r="F76">
         <v>28575887.30375</v>
@@ -4576,7 +4576,7 @@
         <v>0</v>
       </c>
       <c r="E77">
-        <v>0.6956521739130435</v>
+        <v>0.7318840579710145</v>
       </c>
       <c r="F77">
         <v>30872887.30375</v>
@@ -4599,7 +4599,7 @@
         <v>-0.00161</v>
       </c>
       <c r="E78">
-        <v>0.7173913043478261</v>
+        <v>0.7608695652173914</v>
       </c>
       <c r="F78">
         <v>30631387.30375</v>
@@ -4622,7 +4622,7 @@
         <v>-0.005946666666666667</v>
       </c>
       <c r="E79">
-        <v>0.7246376811594203</v>
+        <v>0.7681159420289855</v>
       </c>
       <c r="F79">
         <v>29980887.30375</v>
@@ -4645,7 +4645,7 @@
         <v>0</v>
       </c>
       <c r="E80">
-        <v>0.7391304347826086</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="F80">
         <v>32286887.30375</v>

</xml_diff>